<commit_message>
Interim industry calibration edits
</commit_message>
<xml_diff>
--- a/InputData/indst/BIEEI/BAU Industrial Equipment Efficiency Improvement.xlsx
+++ b/InputData/indst/BIEEI/BAU Industrial Equipment Efficiency Improvement.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr autoCompressPictures="0" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Modeling\EPS\US\eps-us\InputData\indst\BIEEI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\indst\BIEEI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97FCFF07-89CF-42AB-A305-D328A1CD8B0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDD4C56E-14AD-4D97-BB69-02E88EA3EA21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32550" yWindow="3585" windowWidth="24180" windowHeight="11715" tabRatio="770" xr2:uid="{7D5963C0-FA73-4A20-914D-C5C19178119F}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" tabRatio="770" activeTab="1" xr2:uid="{7D5963C0-FA73-4A20-914D-C5C19178119F}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -1710,7 +1710,7 @@
     </row>
     <row r="11" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A11" s="5">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="B11" t="s">
         <v>18</v>
@@ -1833,119 +1833,119 @@
       </c>
       <c r="C16" s="8">
         <f>(1+$A11)^(1/($A13-$A12))-1</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="D16" s="8">
         <f t="shared" ref="D16:AE16" si="1">(1+$A11)^(1/($A13-$A12))-1</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="E16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="F16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="G16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="H16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="I16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="J16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="K16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="L16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="M16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="N16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="O16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="P16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="Q16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="R16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="S16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="T16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="U16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="V16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="W16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="X16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="Y16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="Z16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="AA16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="AB16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="AC16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="AD16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="AE16" s="8">
         <f t="shared" si="1"/>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
     </row>
   </sheetData>
@@ -2069,119 +2069,119 @@
       </c>
       <c r="C2" s="11">
         <f>Calculations!C$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="D2" s="11">
         <f>Calculations!D$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="E2" s="11">
         <f>Calculations!E$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="F2" s="11">
         <f>Calculations!F$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="G2" s="11">
         <f>Calculations!G$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="H2" s="11">
         <f>Calculations!H$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="I2" s="11">
         <f>Calculations!I$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="J2" s="11">
         <f>Calculations!J$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="K2" s="11">
         <f>Calculations!K$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="L2" s="11">
         <f>Calculations!L$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="M2" s="11">
         <f>Calculations!M$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="N2" s="11">
         <f>Calculations!N$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="O2" s="11">
         <f>Calculations!O$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="P2" s="11">
         <f>Calculations!P$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="Q2" s="11">
         <f>Calculations!Q$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="R2" s="11">
         <f>Calculations!R$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="S2" s="11">
         <f>Calculations!S$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="T2" s="11">
         <f>Calculations!T$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="U2" s="11">
         <f>Calculations!U$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="V2" s="11">
         <f>Calculations!V$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="W2" s="11">
         <f>Calculations!W$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="X2" s="11">
         <f>Calculations!X$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="Y2" s="11">
         <f>Calculations!Y$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="Z2" s="11">
         <f>Calculations!Z$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="AA2" s="11">
         <f>Calculations!AA$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="AB2" s="11">
         <f>Calculations!AB$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="AC2" s="11">
         <f>Calculations!AC$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="AD2" s="11">
         <f>Calculations!AD$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="AE2" s="11">
         <f>Calculations!AE$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
     </row>
     <row r="3" spans="1:31" x14ac:dyDescent="0.35">
@@ -2194,119 +2194,119 @@
       </c>
       <c r="C3" s="11">
         <f>Calculations!C$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="D3" s="11">
         <f>Calculations!D$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="E3" s="11">
         <f>Calculations!E$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="F3" s="11">
         <f>Calculations!F$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="G3" s="11">
         <f>Calculations!G$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="H3" s="11">
         <f>Calculations!H$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="I3" s="11">
         <f>Calculations!I$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="J3" s="11">
         <f>Calculations!J$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="K3" s="11">
         <f>Calculations!K$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="L3" s="11">
         <f>Calculations!L$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="M3" s="11">
         <f>Calculations!M$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="N3" s="11">
         <f>Calculations!N$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="O3" s="11">
         <f>Calculations!O$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="P3" s="11">
         <f>Calculations!P$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="Q3" s="11">
         <f>Calculations!Q$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="R3" s="11">
         <f>Calculations!R$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="S3" s="11">
         <f>Calculations!S$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="T3" s="11">
         <f>Calculations!T$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="U3" s="11">
         <f>Calculations!U$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="V3" s="11">
         <f>Calculations!V$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="W3" s="11">
         <f>Calculations!W$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="X3" s="11">
         <f>Calculations!X$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="Y3" s="11">
         <f>Calculations!Y$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="Z3" s="11">
         <f>Calculations!Z$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="AA3" s="11">
         <f>Calculations!AA$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="AB3" s="11">
         <f>Calculations!AB$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="AC3" s="11">
         <f>Calculations!AC$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="AD3" s="11">
         <f>Calculations!AD$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
       <c r="AE3" s="11">
         <f>Calculations!AE$16</f>
-        <v>1.4079754523293353E-2</v>
+        <v>7.724284767762768E-3</v>
       </c>
     </row>
     <row r="4" spans="1:31" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Update efficiency files for mobile equipment
</commit_message>
<xml_diff>
--- a/InputData/indst/BIEEI/BAU Industrial Equipment Efficiency Improvement.xlsx
+++ b/InputData/indst/BIEEI/BAU Industrial Equipment Efficiency Improvement.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr autoCompressPictures="0" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us\InputData\indst\BIEEI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{921C2946-FE8F-481C-BD3E-21564C8285A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9816D59-69FF-47F2-BCF5-DED02AA8EA84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-26580" yWindow="735" windowWidth="25665" windowHeight="15090" tabRatio="770" activeTab="1" xr2:uid="{7D5963C0-FA73-4A20-914D-C5C19178119F}"/>
+    <workbookView xWindow="380" yWindow="380" windowWidth="17790" windowHeight="9120" tabRatio="770" xr2:uid="{7D5963C0-FA73-4A20-914D-C5C19178119F}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -1517,23 +1517,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D20"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="76.5703125" customWidth="1"/>
-    <col min="3" max="3" width="5.140625" customWidth="1"/>
-    <col min="4" max="4" width="57.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="60.42578125" customWidth="1"/>
+    <col min="2" max="2" width="76.54296875" customWidth="1"/>
+    <col min="3" max="3" width="5.1796875" customWidth="1"/>
+    <col min="4" max="4" width="57.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="60.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -1541,67 +1541,67 @@
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B6" s="6">
         <v>2025</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B9" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>4</v>
       </c>
       <c r="D12" s="4"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>5</v>
       </c>
       <c r="D13" s="4"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
       <c r="D14" s="4"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
       <c r="D15" s="4"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
       <c r="D16" s="4"/>
     </row>
-    <row r="17" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D17" s="4"/>
     </row>
-    <row r="18" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D18" s="3"/>
     </row>
-    <row r="19" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D19" s="4"/>
     </row>
-    <row r="20" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="4:4" x14ac:dyDescent="0.35">
       <c r="D20" s="3"/>
     </row>
   </sheetData>
@@ -1618,16 +1618,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54D27B78-5F3A-4024-A428-861147EC67D3}">
   <dimension ref="B18:M28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.81640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="34" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="8.1796875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.26953125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="18" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:13" x14ac:dyDescent="0.35">
       <c r="D18" t="s">
         <v>17</v>
       </c>
@@ -1644,7 +1644,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="19" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B19" t="s">
         <v>29</v>
       </c>
@@ -1676,7 +1676,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="20" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B20" t="s">
         <v>15</v>
       </c>
@@ -1712,7 +1712,7 @@
         <v>5.4215327566901061E-3</v>
       </c>
     </row>
-    <row r="21" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B21" t="s">
         <v>15</v>
       </c>
@@ -1748,7 +1748,7 @@
         <v>1.7331269176886765E-3</v>
       </c>
     </row>
-    <row r="22" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B22" t="s">
         <v>15</v>
       </c>
@@ -1784,7 +1784,7 @@
         <v>5.3439247221002129E-3</v>
       </c>
     </row>
-    <row r="23" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B23" t="s">
         <v>24</v>
       </c>
@@ -1820,7 +1820,7 @@
         <v>2.6967917075848558E-3</v>
       </c>
     </row>
-    <row r="24" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B24" t="s">
         <v>25</v>
       </c>
@@ -1856,7 +1856,7 @@
         <v>5.3233059513549952E-3</v>
       </c>
     </row>
-    <row r="25" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B25" t="s">
         <v>25</v>
       </c>
@@ -1892,7 +1892,7 @@
         <v>2.8308672369490306E-3</v>
       </c>
     </row>
-    <row r="26" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B26" t="s">
         <v>26</v>
       </c>
@@ -1928,7 +1928,7 @@
         <v>4.6608383495440053E-3</v>
       </c>
     </row>
-    <row r="27" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B27" t="s">
         <v>27</v>
       </c>
@@ -1964,7 +1964,7 @@
         <v>4.4855245842795322E-3</v>
       </c>
     </row>
-    <row r="28" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:13" x14ac:dyDescent="0.35">
       <c r="B28" t="s">
         <v>28</v>
       </c>
@@ -2012,12 +2012,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="45.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="45.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -2112,7 +2112,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -2236,7 +2236,7 @@
         <v>1.7331269176886765E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -2360,7 +2360,7 @@
         <v>1.7331269176886765E-3</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -2484,7 +2484,7 @@
         <v>1.7331269176886765E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -2608,7 +2608,7 @@
         <v>1.7331269176886765E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -2732,7 +2732,7 @@
         <v>2.6967917075848558E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -2740,123 +2740,123 @@
         <v>0</v>
       </c>
       <c r="C7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="D7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="E7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="F7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="G7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="H7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="I7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="J7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="K7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="L7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="M7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="N7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="O7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="P7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="Q7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="R7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="S7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="T7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="U7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="V7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="W7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="X7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="Y7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="Z7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="AA7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="AB7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="AC7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="AD7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="AE7" s="15">
-        <f>MECS!$M$24</f>
-        <v>5.3233059513549952E-3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -2980,7 +2980,7 @@
         <v>4.6608383495440053E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -2988,120 +2988,120 @@
         <v>0</v>
       </c>
       <c r="C9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f>C7</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="D9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" ref="D9:AE9" si="0">D7</f>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="E9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="F9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="G9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="H9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="I9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="J9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="K9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="L9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="M9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="N9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="O9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="P9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="Q9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="R9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="S9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="T9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="U9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="V9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="W9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="X9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="Y9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="Z9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="AA9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="AB9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="AC9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="AD9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
       <c r="AE9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>2.8308672369490306E-3</v>
       </c>
     </row>
   </sheetData>
@@ -3115,12 +3115,12 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:AE9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="45.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="45.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -3215,7 +3215,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -3339,7 +3339,7 @@
         <v>5.4215327566901061E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -3463,7 +3463,7 @@
         <v>5.4215327566901061E-3</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -3587,7 +3587,7 @@
         <v>5.4215327566901061E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3711,7 +3711,7 @@
         <v>5.4215327566901061E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -3835,7 +3835,7 @@
         <v>2.6967917075848558E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -3959,7 +3959,7 @@
         <v>5.3233059513549952E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -4083,7 +4083,7 @@
         <v>4.6608383495440053E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -4091,120 +4091,120 @@
         <v>0</v>
       </c>
       <c r="C9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f>C7</f>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="D9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" ref="D9:AE9" si="0">D7</f>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="E9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="F9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="G9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="H9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="I9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="J9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="K9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="L9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="M9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="N9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="O9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="P9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="Q9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="R9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="S9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="T9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="U9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="V9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="W9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="X9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="Y9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="Z9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="AA9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="AB9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="AC9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="AD9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
       <c r="AE9" s="17">
-        <f>MECS!$M$28</f>
-        <v>2.726215022795353E-3</v>
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adds nonprocess end uses to industry energy consumption
</commit_message>
<xml_diff>
--- a/InputData/indst/BIEEI/BAU Industrial Equipment Efficiency Improvement.xlsx
+++ b/InputData/indst/BIEEI/BAU Industrial Equipment Efficiency Improvement.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr autoCompressPictures="0" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us\InputData\indst\BIEEI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9816D59-69FF-47F2-BCF5-DED02AA8EA84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C06D2ECF-705D-479E-A615-D7327B296E28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="380" windowWidth="17790" windowHeight="9120" tabRatio="770" xr2:uid="{7D5963C0-FA73-4A20-914D-C5C19178119F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="770" activeTab="4" xr2:uid="{7D5963C0-FA73-4A20-914D-C5C19178119F}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
     <sheet name="MECS" sheetId="149" r:id="rId2"/>
-    <sheet name="BIEEI-elec" sheetId="146" r:id="rId3"/>
-    <sheet name="BIEEI-other" sheetId="148" r:id="rId4"/>
+    <sheet name="lighting" sheetId="150" r:id="rId3"/>
+    <sheet name="BIEEI-elec" sheetId="146" r:id="rId4"/>
+    <sheet name="BIEEI-other" sheetId="148" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -55,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="42">
   <si>
     <t>Sources:</t>
   </si>
@@ -91,9 +92,6 @@
   </si>
   <si>
     <t>Machine Drive</t>
-  </si>
-  <si>
-    <t>Electrochem</t>
   </si>
   <si>
     <t>Other process</t>
@@ -169,6 +167,21 @@
   </si>
   <si>
     <t>improvement</t>
+  </si>
+  <si>
+    <t>Facility HVAC</t>
+  </si>
+  <si>
+    <t>Facility lighting</t>
+  </si>
+  <si>
+    <t>Other nonprocess</t>
+  </si>
+  <si>
+    <t>start year lighting efficiency from SYIEUEFbIPaF</t>
+  </si>
+  <si>
+    <t>assumed efficiency 2050 (all LEDs)</t>
   </si>
 </sst>
 </file>
@@ -392,7 +405,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="39">
+  <fills count="40">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -605,6 +618,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -995,7 +1014,7 @@
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -1019,7 +1038,8 @@
     <xf numFmtId="166" fontId="0" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="166" fontId="0" fillId="36" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="166" fontId="0" fillId="37" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="166" fontId="0" fillId="38" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="39" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="106">
     <cellStyle name="20% - Accent1" xfId="43" builtinId="30" customBuiltin="1"/>
@@ -1517,91 +1537,91 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D20"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="76.54296875" customWidth="1"/>
-    <col min="3" max="3" width="5.1796875" customWidth="1"/>
-    <col min="4" max="4" width="57.81640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="60.453125" customWidth="1"/>
+    <col min="2" max="2" width="76.5703125" customWidth="1"/>
+    <col min="3" max="3" width="5.140625" customWidth="1"/>
+    <col min="4" max="4" width="57.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="60.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B6" s="6">
         <v>2025</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B8" t="s">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="B9" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>4</v>
       </c>
       <c r="D12" s="4"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>5</v>
       </c>
       <c r="D13" s="4"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D14" s="4"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D15" s="4"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="D16" s="4"/>
     </row>
-    <row r="17" spans="4:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D17" s="4"/>
     </row>
-    <row r="18" spans="4:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D18" s="3"/>
     </row>
-    <row r="19" spans="4:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D19" s="4"/>
     </row>
-    <row r="20" spans="4:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="4:4" x14ac:dyDescent="0.25">
       <c r="D20" s="3"/>
     </row>
   </sheetData>
@@ -1618,21 +1638,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54D27B78-5F3A-4024-A428-861147EC67D3}">
   <dimension ref="B18:M28"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="15.453125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="34" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="8.1796875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="18" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="18" spans="2:13" x14ac:dyDescent="0.25">
       <c r="D18" t="s">
+        <v>16</v>
+      </c>
+      <c r="E18" t="s">
         <v>17</v>
-      </c>
-      <c r="E18" t="s">
-        <v>18</v>
       </c>
       <c r="F18">
         <v>2018</v>
@@ -1641,27 +1661,27 @@
         <v>2050</v>
       </c>
       <c r="K18" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="19" spans="2:13" x14ac:dyDescent="0.35">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
+        <v>28</v>
+      </c>
+      <c r="C19" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" t="s">
+        <v>19</v>
+      </c>
+      <c r="E19" t="s">
+        <v>20</v>
+      </c>
+      <c r="F19" t="s">
         <v>29</v>
       </c>
-      <c r="C19" t="s">
-        <v>19</v>
-      </c>
-      <c r="D19" t="s">
-        <v>20</v>
-      </c>
-      <c r="E19" t="s">
-        <v>21</v>
-      </c>
-      <c r="F19" t="s">
-        <v>30</v>
-      </c>
       <c r="G19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I19">
         <v>2021</v>
@@ -1670,18 +1690,18 @@
         <v>2050</v>
       </c>
       <c r="K19" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="M19" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B20" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="20" spans="2:13" x14ac:dyDescent="0.35">
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>15</v>
-      </c>
-      <c r="C20" t="s">
-        <v>16</v>
       </c>
       <c r="D20">
         <v>0.218</v>
@@ -1712,12 +1732,12 @@
         <v>5.4215327566901061E-3</v>
       </c>
     </row>
-    <row r="21" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B21" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C21" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D21">
         <v>2.1999999999999999E-2</v>
@@ -1748,12 +1768,12 @@
         <v>1.7331269176886765E-3</v>
       </c>
     </row>
-    <row r="22" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="22" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C22" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D22">
         <v>0.20399999999999999</v>
@@ -1784,12 +1804,12 @@
         <v>5.3439247221002129E-3</v>
       </c>
     </row>
-    <row r="23" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C23" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D23">
         <v>3.9E-2</v>
@@ -1820,12 +1840,12 @@
         <v>2.6967917075848558E-3</v>
       </c>
     </row>
-    <row r="24" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="24" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C24" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D24">
         <v>1.2999999999999999E-2</v>
@@ -1856,12 +1876,12 @@
         <v>5.3233059513549952E-3</v>
       </c>
     </row>
-    <row r="25" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="25" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C25" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D25">
         <v>0.19900000000000001</v>
@@ -1892,12 +1912,12 @@
         <v>2.8308672369490306E-3</v>
       </c>
     </row>
-    <row r="26" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="26" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B26" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C26" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D26">
         <v>1E-3</v>
@@ -1928,12 +1948,12 @@
         <v>4.6608383495440053E-3</v>
       </c>
     </row>
-    <row r="27" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B27" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C27" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D27">
         <v>1.0999999999999999E-2</v>
@@ -1964,12 +1984,12 @@
         <v>4.4855245842795322E-3</v>
       </c>
     </row>
-    <row r="28" spans="2:13" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B28" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C28" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D28">
         <v>7.0000000000000001E-3</v>
@@ -2007,1101 +2027,61 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BF4B172-C1A6-434D-B033-E39FCD33B2CE}">
-  <sheetPr>
-    <tabColor theme="3"/>
-  </sheetPr>
-  <dimension ref="A1:AE9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA830FA0-061B-47E2-AAB7-CBEAD2743A6E}">
+  <dimension ref="B5:F14"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="45.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1">
-        <v>2021</v>
-      </c>
-      <c r="C1">
-        <v>2022</v>
-      </c>
-      <c r="D1">
-        <v>2023</v>
-      </c>
-      <c r="E1">
+    <row r="5" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B5">
         <v>2024</v>
       </c>
-      <c r="F1">
-        <v>2025</v>
-      </c>
-      <c r="G1">
-        <v>2026</v>
-      </c>
-      <c r="H1">
-        <v>2027</v>
-      </c>
-      <c r="I1">
-        <v>2028</v>
-      </c>
-      <c r="J1">
-        <v>2029</v>
-      </c>
-      <c r="K1">
-        <v>2030</v>
-      </c>
-      <c r="L1">
-        <v>2031</v>
-      </c>
-      <c r="M1">
-        <v>2032</v>
-      </c>
-      <c r="N1">
-        <v>2033</v>
-      </c>
-      <c r="O1">
-        <v>2034</v>
-      </c>
-      <c r="P1">
-        <v>2035</v>
-      </c>
-      <c r="Q1">
-        <v>2036</v>
-      </c>
-      <c r="R1">
-        <v>2037</v>
-      </c>
-      <c r="S1">
-        <v>2038</v>
-      </c>
-      <c r="T1">
-        <v>2039</v>
-      </c>
-      <c r="U1">
-        <v>2040</v>
-      </c>
-      <c r="V1">
-        <v>2041</v>
-      </c>
-      <c r="W1">
-        <v>2042</v>
-      </c>
-      <c r="X1">
-        <v>2043</v>
-      </c>
-      <c r="Y1">
-        <v>2044</v>
-      </c>
-      <c r="Z1">
-        <v>2045</v>
-      </c>
-      <c r="AA1">
-        <v>2046</v>
-      </c>
-      <c r="AB1">
-        <v>2047</v>
-      </c>
-      <c r="AC1">
-        <v>2048</v>
-      </c>
-      <c r="AD1">
-        <v>2049</v>
-      </c>
-      <c r="AE1">
+      <c r="C5">
+        <v>0.85307500000000003</v>
+      </c>
+      <c r="D5">
+        <f>1/C5</f>
+        <v>1.1722298742783459</v>
+      </c>
+      <c r="E5" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="6" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B6">
         <v>2050</v>
       </c>
-    </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="8">
-        <v>0</v>
-      </c>
-      <c r="C2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="D2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="E2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="F2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="G2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="H2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="I2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="J2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="K2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="L2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="M2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="N2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="O2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="P2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="Q2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="R2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="S2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="T2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="U2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="V2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="W2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="X2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="Y2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="Z2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="AA2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="AB2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="AC2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="AD2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="AE2" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="8">
-        <v>0</v>
-      </c>
-      <c r="C3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="D3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="E3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="F3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="G3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="H3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="I3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="J3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="K3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="L3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="M3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="N3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="O3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="P3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="Q3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="R3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="S3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="T3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="U3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="V3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="W3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="X3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="Y3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="Z3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="AA3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="AB3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="AC3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="AD3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="AE3" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" s="8">
-        <v>0</v>
-      </c>
-      <c r="C4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="D4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="E4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="F4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="G4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="H4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="I4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="J4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="K4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="L4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="M4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="N4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="O4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="P4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="Q4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="R4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="S4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="T4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="U4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="V4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="W4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="X4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="Y4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="Z4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="AA4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="AB4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="AC4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="AD4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="AE4" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5" s="8">
-        <v>0</v>
-      </c>
-      <c r="C5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="D5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="E5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="F5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="G5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="H5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="I5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="J5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="K5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="L5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="M5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="N5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="O5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="P5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="Q5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="R5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="S5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="T5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="U5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="V5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="W5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="X5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="Y5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="Z5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="AA5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="AB5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="AC5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="AD5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-      <c r="AE5" s="13">
-        <f>MECS!$M$21</f>
-        <v>1.7331269176886765E-3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="9">
-        <v>0</v>
-      </c>
-      <c r="C6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="D6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="E6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="F6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="G6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="H6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="I6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="J6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="K6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="L6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="M6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="N6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="O6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="P6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="Q6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="R6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="S6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="T6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="U6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="V6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="W6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="X6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="Y6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="Z6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="AA6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="AB6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="AC6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="AD6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-      <c r="AE6" s="14">
-        <f>MECS!$M$23</f>
-        <v>2.6967917075848558E-3</v>
-      </c>
-    </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="10">
-        <v>0</v>
-      </c>
-      <c r="C7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="D7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="E7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="F7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="G7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="H7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="I7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="J7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="K7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="L7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="M7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="N7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="O7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="P7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="Q7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="R7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="S7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="T7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="U7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="V7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="W7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="X7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="Y7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="Z7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="AA7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="AB7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="AC7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="AD7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="AE7" s="15">
-        <f>MECS!$M$25</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-    </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" s="11">
-        <v>0</v>
-      </c>
-      <c r="C8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="D8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="E8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="F8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="G8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="H8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="I8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="J8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="K8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="L8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="M8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="N8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="O8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="P8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="Q8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="R8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="S8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="T8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="U8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="V8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="W8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="X8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="Y8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="Z8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="AA8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="AB8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="AC8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="AD8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-      <c r="AE8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" s="12">
-        <v>0</v>
-      </c>
-      <c r="C9" s="17">
-        <f>C7</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="D9" s="17">
-        <f t="shared" ref="D9:AE9" si="0">D7</f>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="E9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="F9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="G9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="H9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="I9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="J9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="K9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="L9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="M9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="N9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="O9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="P9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="Q9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="R9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="S9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="T9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="U9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="V9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="W9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="X9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="Y9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="Z9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="AA9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="AB9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="AC9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="AD9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
-      </c>
-      <c r="AE9" s="17">
-        <f t="shared" si="0"/>
-        <v>2.8308672369490306E-3</v>
+      <c r="C6" s="17">
+        <v>0.9</v>
+      </c>
+      <c r="D6">
+        <f>1/C6</f>
+        <v>1.1111111111111112</v>
+      </c>
+      <c r="E6" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="D8">
+        <f>1-D6/D5</f>
+        <v>5.2138888888888735E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="F9">
+        <f>D8/25</f>
+        <v>2.0855555555555493E-3</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="D14" s="7">
+        <f>1-(1-D8)^(1/($B$6-$B$5))</f>
+        <v>2.0573919973707611E-3</v>
       </c>
     </row>
   </sheetData>
@@ -3110,17 +2090,1371 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BF4B172-C1A6-434D-B033-E39FCD33B2CE}">
+  <sheetPr>
+    <tabColor theme="3"/>
+  </sheetPr>
+  <dimension ref="A1:AE11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="45.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1">
+        <v>2021</v>
+      </c>
+      <c r="C1">
+        <v>2022</v>
+      </c>
+      <c r="D1">
+        <v>2023</v>
+      </c>
+      <c r="E1">
+        <v>2024</v>
+      </c>
+      <c r="F1">
+        <v>2025</v>
+      </c>
+      <c r="G1">
+        <v>2026</v>
+      </c>
+      <c r="H1">
+        <v>2027</v>
+      </c>
+      <c r="I1">
+        <v>2028</v>
+      </c>
+      <c r="J1">
+        <v>2029</v>
+      </c>
+      <c r="K1">
+        <v>2030</v>
+      </c>
+      <c r="L1">
+        <v>2031</v>
+      </c>
+      <c r="M1">
+        <v>2032</v>
+      </c>
+      <c r="N1">
+        <v>2033</v>
+      </c>
+      <c r="O1">
+        <v>2034</v>
+      </c>
+      <c r="P1">
+        <v>2035</v>
+      </c>
+      <c r="Q1">
+        <v>2036</v>
+      </c>
+      <c r="R1">
+        <v>2037</v>
+      </c>
+      <c r="S1">
+        <v>2038</v>
+      </c>
+      <c r="T1">
+        <v>2039</v>
+      </c>
+      <c r="U1">
+        <v>2040</v>
+      </c>
+      <c r="V1">
+        <v>2041</v>
+      </c>
+      <c r="W1">
+        <v>2042</v>
+      </c>
+      <c r="X1">
+        <v>2043</v>
+      </c>
+      <c r="Y1">
+        <v>2044</v>
+      </c>
+      <c r="Z1">
+        <v>2045</v>
+      </c>
+      <c r="AA1">
+        <v>2046</v>
+      </c>
+      <c r="AB1">
+        <v>2047</v>
+      </c>
+      <c r="AC1">
+        <v>2048</v>
+      </c>
+      <c r="AD1">
+        <v>2049</v>
+      </c>
+      <c r="AE1">
+        <v>2050</v>
+      </c>
+    </row>
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="8">
+        <v>0</v>
+      </c>
+      <c r="C2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="D2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="E2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="F2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="G2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="H2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="I2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="J2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="K2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="L2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="M2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="N2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="O2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="P2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="Q2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="R2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="S2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="T2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="U2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="V2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="W2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="X2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="Y2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="Z2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="AA2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="AB2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="AC2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="AD2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="AE2" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="8">
+        <v>0</v>
+      </c>
+      <c r="C3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="D3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="E3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="F3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="G3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="H3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="I3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="J3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="K3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="L3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="M3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="N3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="O3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="P3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="Q3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="R3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="S3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="T3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="U3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="V3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="W3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="X3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="Y3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="Z3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="AA3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="AB3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="AC3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="AD3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="AE3" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="8">
+        <v>0</v>
+      </c>
+      <c r="C4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="D4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="E4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="F4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="G4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="H4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="I4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="J4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="K4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="L4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="M4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="N4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="O4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="P4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="Q4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="R4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="S4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="T4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="U4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="V4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="W4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="X4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="Y4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="Z4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="AA4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="AB4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="AC4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="AD4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="AE4" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="8">
+        <v>0</v>
+      </c>
+      <c r="C5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="D5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="E5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="F5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="G5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="H5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="I5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="J5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="K5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="L5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="M5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="N5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="O5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="P5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="Q5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="R5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="S5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="T5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="U5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="V5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="W5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="X5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="Y5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="Z5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="AA5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="AB5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="AC5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="AD5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="AE5" s="13">
+        <f>MECS!$M$21</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="9">
+        <v>0</v>
+      </c>
+      <c r="C6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="D6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="E6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="F6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="G6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="H6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="I6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="J6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="K6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="L6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="M6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="N6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="O6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="P6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="Q6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="R6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="S6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="T6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="U6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="V6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="W6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="X6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="Y6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="Z6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="AA6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="AB6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="AC6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="AD6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+      <c r="AE6" s="14">
+        <f>MECS!$M$23</f>
+        <v>2.6967917075848558E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="10">
+        <v>0</v>
+      </c>
+      <c r="C7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="D7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="E7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="F7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="G7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="H7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="I7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="J7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="K7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="L7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="M7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="N7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="O7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="P7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="Q7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="R7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="S7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="T7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="U7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="V7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="W7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="X7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="Y7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="Z7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="AA7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="AB7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="AC7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="AD7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+      <c r="AE7" s="15">
+        <f>MECS!$M$25</f>
+        <v>2.8308672369490306E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="11">
+        <v>0</v>
+      </c>
+      <c r="C8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="D8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="E8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="F8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="G8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="H8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="I8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="J8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="K8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="L8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="M8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="N8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="O8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="P8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="Q8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="R8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="S8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="T8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="U8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="V8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="W8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="X8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="Y8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="Z8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="AA8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="AB8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="AC8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="AD8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+      <c r="AE8" s="16">
+        <f>AVERAGE(MECS!$M$28,MECS!$M$26)</f>
+        <v>3.6935266861696792E-3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" s="8">
+        <f>B2</f>
+        <v>0</v>
+      </c>
+      <c r="C9" s="8">
+        <f t="shared" ref="C9:AE10" si="0">C2</f>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="D9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="E9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="F9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="G9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="H9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="I9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="J9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="K9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="L9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="M9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="N9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="O9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="P9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="Q9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="R9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="S9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="T9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="U9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="V9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="W9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="X9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="Y9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="Z9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="AA9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="AB9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="AC9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="AD9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+      <c r="AE9" s="8">
+        <f t="shared" si="0"/>
+        <v>1.7331269176886765E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="12">
+        <f>B3</f>
+        <v>0</v>
+      </c>
+      <c r="C10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="D10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="E10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="F10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="G10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="H10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="I10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="J10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="K10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="L10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="M10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="N10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="O10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="P10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="Q10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="R10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="S10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="T10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="U10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="V10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="W10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="X10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="Y10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="Z10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="AA10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="AB10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="AC10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="AD10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="AE10" s="12">
+        <f>lighting!$D$14</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11" s="18">
+        <f>AVERAGE(B2:B10)</f>
+        <v>0</v>
+      </c>
+      <c r="C11" s="18">
+        <f t="shared" ref="C11:AE11" si="1">AVERAGE(C2:C10)</f>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="D11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="E11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="F11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="G11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="H11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="I11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="J11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="K11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="L11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="M11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="N11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="O11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="P11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="Q11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="R11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="S11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="T11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="U11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="V11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="W11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="X11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="Y11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="Z11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="AA11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="AB11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="AC11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="AD11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+      <c r="AE11" s="18">
+        <f t="shared" si="1"/>
+        <v>2.216023579613079E-3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15C4D4F2-9192-4557-9476-0BAD41DB5078}">
   <sheetPr>
     <tabColor theme="3"/>
   </sheetPr>
-  <dimension ref="A1:AE9"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AE11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="45.453125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="45.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -3215,7 +3549,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -3339,7 +3673,7 @@
         <v>5.4215327566901061E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -3463,7 +3797,7 @@
         <v>5.4215327566901061E-3</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -3587,7 +3921,7 @@
         <v>5.4215327566901061E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -3711,7 +4045,7 @@
         <v>5.4215327566901061E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>10</v>
       </c>
@@ -3835,7 +4169,7 @@
         <v>2.6967917075848558E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -3959,7 +4293,7 @@
         <v>5.3233059513549952E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>12</v>
       </c>
@@ -3967,244 +4301,494 @@
         <v>0</v>
       </c>
       <c r="C8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="D8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="E8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="F8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="G8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="H8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="I8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="J8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="K8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="L8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="M8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="N8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="O8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="P8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="Q8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="R8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="S8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="T8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="U8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="V8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="W8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="X8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="Y8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="Z8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="AA8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="AB8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="AC8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="AD8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
       </c>
       <c r="AE8" s="16">
-        <f>MECS!$M$26</f>
-        <v>4.6608383495440053E-3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.35">
+        <f>MECS!$M$27</f>
+        <v>4.4855245842795322E-3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" s="12">
+        <v>37</v>
+      </c>
+      <c r="B9" s="13">
         <v>0</v>
       </c>
-      <c r="C9" s="17">
+      <c r="C9" s="13">
         <f>C7</f>
         <v>5.3233059513549952E-3</v>
       </c>
-      <c r="D9" s="17">
+      <c r="D9" s="13">
         <f t="shared" ref="D9:AE9" si="0">D7</f>
         <v>5.3233059513549952E-3</v>
       </c>
-      <c r="E9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
-      </c>
-      <c r="F9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
-      </c>
-      <c r="G9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
-      </c>
-      <c r="H9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
-      </c>
-      <c r="I9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
-      </c>
-      <c r="J9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
-      </c>
-      <c r="K9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
-      </c>
-      <c r="L9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
-      </c>
-      <c r="M9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
-      </c>
-      <c r="N9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
-      </c>
-      <c r="O9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
-      </c>
-      <c r="P9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
-      </c>
-      <c r="Q9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
-      </c>
-      <c r="R9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
-      </c>
-      <c r="S9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
-      </c>
-      <c r="T9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
-      </c>
-      <c r="U9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
-      </c>
-      <c r="V9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
-      </c>
-      <c r="W9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
-      </c>
-      <c r="X9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
-      </c>
-      <c r="Y9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
-      </c>
-      <c r="Z9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
-      </c>
-      <c r="AA9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
-      </c>
-      <c r="AB9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
-      </c>
-      <c r="AC9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
-      </c>
-      <c r="AD9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
-      </c>
-      <c r="AE9" s="17">
-        <f t="shared" si="0"/>
-        <v>5.3233059513549952E-3</v>
+      <c r="E9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+      <c r="F9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+      <c r="G9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+      <c r="H9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+      <c r="I9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+      <c r="J9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+      <c r="K9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+      <c r="L9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+      <c r="M9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+      <c r="N9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+      <c r="O9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+      <c r="P9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+      <c r="Q9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+      <c r="R9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+      <c r="S9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+      <c r="T9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+      <c r="U9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+      <c r="V9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+      <c r="W9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+      <c r="X9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+      <c r="Y9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+      <c r="Z9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+      <c r="AA9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+      <c r="AB9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+      <c r="AC9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+      <c r="AD9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+      <c r="AE9" s="13">
+        <f t="shared" si="0"/>
+        <v>5.3233059513549952E-3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="12">
+        <f>'BIEEI-elec'!B10</f>
+        <v>0</v>
+      </c>
+      <c r="C10" s="12">
+        <f>'BIEEI-elec'!C10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="D10" s="12">
+        <f>'BIEEI-elec'!D10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="E10" s="12">
+        <f>'BIEEI-elec'!E10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="F10" s="12">
+        <f>'BIEEI-elec'!F10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="G10" s="12">
+        <f>'BIEEI-elec'!G10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="H10" s="12">
+        <f>'BIEEI-elec'!H10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="I10" s="12">
+        <f>'BIEEI-elec'!I10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="J10" s="12">
+        <f>'BIEEI-elec'!J10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="K10" s="12">
+        <f>'BIEEI-elec'!K10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="L10" s="12">
+        <f>'BIEEI-elec'!L10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="M10" s="12">
+        <f>'BIEEI-elec'!M10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="N10" s="12">
+        <f>'BIEEI-elec'!N10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="O10" s="12">
+        <f>'BIEEI-elec'!O10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="P10" s="12">
+        <f>'BIEEI-elec'!P10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="Q10" s="12">
+        <f>'BIEEI-elec'!Q10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="R10" s="12">
+        <f>'BIEEI-elec'!R10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="S10" s="12">
+        <f>'BIEEI-elec'!S10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="T10" s="12">
+        <f>'BIEEI-elec'!T10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="U10" s="12">
+        <f>'BIEEI-elec'!U10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="V10" s="12">
+        <f>'BIEEI-elec'!V10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="W10" s="12">
+        <f>'BIEEI-elec'!W10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="X10" s="12">
+        <f>'BIEEI-elec'!X10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="Y10" s="12">
+        <f>'BIEEI-elec'!Y10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="Z10" s="12">
+        <f>'BIEEI-elec'!Z10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="AA10" s="12">
+        <f>'BIEEI-elec'!AA10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="AB10" s="12">
+        <f>'BIEEI-elec'!AB10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="AC10" s="12">
+        <f>'BIEEI-elec'!AC10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="AD10" s="12">
+        <f>'BIEEI-elec'!AD10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+      <c r="AE10" s="12">
+        <f>'BIEEI-elec'!AE10</f>
+        <v>2.0573919973707611E-3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:31" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>39</v>
+      </c>
+      <c r="B11" s="18">
+        <f>AVERAGE(B2:B10)</f>
+        <v>0</v>
+      </c>
+      <c r="C11" s="18">
+        <f t="shared" ref="C11:AE11" si="1">AVERAGE(C2:C10)</f>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="D11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="E11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="F11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="G11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="H11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="I11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="J11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="K11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="L11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="M11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="N11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="O11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="P11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="Q11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="R11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="S11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="T11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="U11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="V11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="W11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="X11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="Y11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="Z11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="AA11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="AB11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="AC11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="AD11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
+      </c>
+      <c r="AE11" s="18">
+        <f t="shared" si="1"/>
+        <v>4.6191612465228404E-3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>